<commit_message>
Conditioning air feed to FBR
</commit_message>
<xml_diff>
--- a/process_sim/results/stream_results.xlsx
+++ b/process_sim/results/stream_results.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F113"/>
+  <dimension ref="A1:F114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3094,7 +3094,7 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>414</v>
+        <v>298.15</v>
       </c>
       <c r="C111" t="n">
         <v>100000</v>
@@ -3114,31 +3114,31 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>F-8</t>
+          <t>F-73T</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>298.15</v>
+        <v>475</v>
       </c>
       <c r="C112" t="n">
         <v>100000</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>G</t>
         </is>
       </c>
       <c r="E112" t="n">
-        <v>8.814462000000001</v>
+        <v>4.17976</v>
       </c>
       <c r="F112" t="n">
-        <v>1849.908327</v>
+        <v>121.859939</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>F-9</t>
+          <t>F-8</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -3153,9 +3153,33 @@
         </is>
       </c>
       <c r="E113" t="n">
+        <v>8.814462000000001</v>
+      </c>
+      <c r="F113" t="n">
+        <v>1849.908327</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>F-9</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>298.15</v>
+      </c>
+      <c r="C114" t="n">
+        <v>100000</v>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E114" t="n">
         <v>0.881446</v>
       </c>
-      <c r="F113" t="n">
+      <c r="F114" t="n">
         <v>16.463097</v>
       </c>
     </row>
@@ -3170,7 +3194,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ113"/>
+  <dimension ref="A1:AQ114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -18068,7 +18092,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>F-8</t>
+          <t>F-73T</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -18135,10 +18159,10 @@
         <v>0</v>
       </c>
       <c r="W112" t="n">
-        <v>0</v>
+        <v>2.982937</v>
       </c>
       <c r="X112" t="n">
-        <v>0</v>
+        <v>1.196823</v>
       </c>
       <c r="Y112" t="n">
         <v>0</v>
@@ -18147,10 +18171,10 @@
         <v>0</v>
       </c>
       <c r="AA112" t="n">
-        <v>1.71857377</v>
+        <v>0</v>
       </c>
       <c r="AB112" t="n">
-        <v>6.27751246</v>
+        <v>0</v>
       </c>
       <c r="AC112" t="n">
         <v>0</v>
@@ -18159,13 +18183,13 @@
         <v>0</v>
       </c>
       <c r="AE112" t="n">
-        <v>0.80980442</v>
+        <v>0</v>
       </c>
       <c r="AF112" t="n">
-        <v>0.00710324</v>
+        <v>0</v>
       </c>
       <c r="AG112" t="n">
-        <v>0.00036732</v>
+        <v>0</v>
       </c>
       <c r="AH112" t="n">
         <v>0</v>
@@ -18189,7 +18213,7 @@
         <v>0</v>
       </c>
       <c r="AO112" t="n">
-        <v>0.00110122</v>
+        <v>0</v>
       </c>
       <c r="AP112" t="n">
         <v>0</v>
@@ -18201,133 +18225,266 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
+          <t>F-8</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>0</v>
+      </c>
+      <c r="C113" t="n">
+        <v>0</v>
+      </c>
+      <c r="D113" t="n">
+        <v>0</v>
+      </c>
+      <c r="E113" t="n">
+        <v>0</v>
+      </c>
+      <c r="F113" t="n">
+        <v>0</v>
+      </c>
+      <c r="G113" t="n">
+        <v>0</v>
+      </c>
+      <c r="H113" t="n">
+        <v>0</v>
+      </c>
+      <c r="I113" t="n">
+        <v>0</v>
+      </c>
+      <c r="J113" t="n">
+        <v>0</v>
+      </c>
+      <c r="K113" t="n">
+        <v>0</v>
+      </c>
+      <c r="L113" t="n">
+        <v>0</v>
+      </c>
+      <c r="M113" t="n">
+        <v>0</v>
+      </c>
+      <c r="N113" t="n">
+        <v>0</v>
+      </c>
+      <c r="O113" t="n">
+        <v>0</v>
+      </c>
+      <c r="P113" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q113" t="n">
+        <v>0</v>
+      </c>
+      <c r="R113" t="n">
+        <v>0</v>
+      </c>
+      <c r="S113" t="n">
+        <v>0</v>
+      </c>
+      <c r="T113" t="n">
+        <v>0</v>
+      </c>
+      <c r="U113" t="n">
+        <v>0</v>
+      </c>
+      <c r="V113" t="n">
+        <v>0</v>
+      </c>
+      <c r="W113" t="n">
+        <v>0</v>
+      </c>
+      <c r="X113" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y113" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA113" t="n">
+        <v>1.71857377</v>
+      </c>
+      <c r="AB113" t="n">
+        <v>6.27751246</v>
+      </c>
+      <c r="AC113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE113" t="n">
+        <v>0.80980442</v>
+      </c>
+      <c r="AF113" t="n">
+        <v>0.00710324</v>
+      </c>
+      <c r="AG113" t="n">
+        <v>0.00036732</v>
+      </c>
+      <c r="AH113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO113" t="n">
+        <v>0.00110122</v>
+      </c>
+      <c r="AP113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ113" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
           <t>F-9</t>
         </is>
       </c>
-      <c r="B113" t="n">
-        <v>0</v>
-      </c>
-      <c r="C113" t="n">
-        <v>0</v>
-      </c>
-      <c r="D113" t="n">
-        <v>0</v>
-      </c>
-      <c r="E113" t="n">
-        <v>0</v>
-      </c>
-      <c r="F113" t="n">
-        <v>0</v>
-      </c>
-      <c r="G113" t="n">
-        <v>0</v>
-      </c>
-      <c r="H113" t="n">
-        <v>0</v>
-      </c>
-      <c r="I113" t="n">
-        <v>0</v>
-      </c>
-      <c r="J113" t="n">
-        <v>0</v>
-      </c>
-      <c r="K113" t="n">
-        <v>0</v>
-      </c>
-      <c r="L113" t="n">
-        <v>0</v>
-      </c>
-      <c r="M113" t="n">
-        <v>0</v>
-      </c>
-      <c r="N113" t="n">
-        <v>0</v>
-      </c>
-      <c r="O113" t="n">
-        <v>0</v>
-      </c>
-      <c r="P113" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q113" t="n">
-        <v>0</v>
-      </c>
-      <c r="R113" t="n">
-        <v>0</v>
-      </c>
-      <c r="S113" t="n">
+      <c r="B114" t="n">
+        <v>0</v>
+      </c>
+      <c r="C114" t="n">
+        <v>0</v>
+      </c>
+      <c r="D114" t="n">
+        <v>0</v>
+      </c>
+      <c r="E114" t="n">
+        <v>0</v>
+      </c>
+      <c r="F114" t="n">
+        <v>0</v>
+      </c>
+      <c r="G114" t="n">
+        <v>0</v>
+      </c>
+      <c r="H114" t="n">
+        <v>0</v>
+      </c>
+      <c r="I114" t="n">
+        <v>0</v>
+      </c>
+      <c r="J114" t="n">
+        <v>0</v>
+      </c>
+      <c r="K114" t="n">
+        <v>0</v>
+      </c>
+      <c r="L114" t="n">
+        <v>0</v>
+      </c>
+      <c r="M114" t="n">
+        <v>0</v>
+      </c>
+      <c r="N114" t="n">
+        <v>0</v>
+      </c>
+      <c r="O114" t="n">
+        <v>0</v>
+      </c>
+      <c r="P114" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q114" t="n">
+        <v>0</v>
+      </c>
+      <c r="R114" t="n">
+        <v>0</v>
+      </c>
+      <c r="S114" t="n">
         <v>0.86953481</v>
       </c>
-      <c r="T113" t="n">
+      <c r="T114" t="n">
         <v>0.00794096</v>
       </c>
-      <c r="U113" t="n">
-        <v>0</v>
-      </c>
-      <c r="V113" t="n">
-        <v>0</v>
-      </c>
-      <c r="W113" t="n">
-        <v>0</v>
-      </c>
-      <c r="X113" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y113" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC113" t="n">
+      <c r="U114" t="n">
+        <v>0</v>
+      </c>
+      <c r="V114" t="n">
+        <v>0</v>
+      </c>
+      <c r="W114" t="n">
+        <v>0</v>
+      </c>
+      <c r="X114" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y114" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC114" t="n">
         <v>0.00397048</v>
       </c>
-      <c r="AD113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ113" t="n">
+      <c r="AD114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ114" t="n">
         <v>0</v>
       </c>
     </row>
@@ -18342,7 +18499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ113"/>
+  <dimension ref="A1:AQ114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -33240,7 +33397,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>F-8</t>
+          <t>F-73T</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -33307,10 +33464,10 @@
         <v>0</v>
       </c>
       <c r="W112" t="n">
-        <v>0</v>
+        <v>0.71366227</v>
       </c>
       <c r="X112" t="n">
-        <v>0</v>
+        <v>0.28633773</v>
       </c>
       <c r="Y112" t="n">
         <v>0</v>
@@ -33319,10 +33476,10 @@
         <v>0</v>
       </c>
       <c r="AA112" t="n">
-        <v>0.19497205</v>
+        <v>0</v>
       </c>
       <c r="AB112" t="n">
-        <v>0.71218324</v>
+        <v>0</v>
       </c>
       <c r="AC112" t="n">
         <v>0</v>
@@ -33331,13 +33488,13 @@
         <v>0</v>
       </c>
       <c r="AE112" t="n">
-        <v>0.09187223999999999</v>
+        <v>0</v>
       </c>
       <c r="AF112" t="n">
-        <v>0.00080586</v>
+        <v>0</v>
       </c>
       <c r="AG112" t="n">
-        <v>4.167e-05</v>
+        <v>0</v>
       </c>
       <c r="AH112" t="n">
         <v>0</v>
@@ -33361,7 +33518,7 @@
         <v>0</v>
       </c>
       <c r="AO112" t="n">
-        <v>0.00012493</v>
+        <v>0</v>
       </c>
       <c r="AP112" t="n">
         <v>0</v>
@@ -33373,133 +33530,266 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
+          <t>F-8</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>0</v>
+      </c>
+      <c r="C113" t="n">
+        <v>0</v>
+      </c>
+      <c r="D113" t="n">
+        <v>0</v>
+      </c>
+      <c r="E113" t="n">
+        <v>0</v>
+      </c>
+      <c r="F113" t="n">
+        <v>0</v>
+      </c>
+      <c r="G113" t="n">
+        <v>0</v>
+      </c>
+      <c r="H113" t="n">
+        <v>0</v>
+      </c>
+      <c r="I113" t="n">
+        <v>0</v>
+      </c>
+      <c r="J113" t="n">
+        <v>0</v>
+      </c>
+      <c r="K113" t="n">
+        <v>0</v>
+      </c>
+      <c r="L113" t="n">
+        <v>0</v>
+      </c>
+      <c r="M113" t="n">
+        <v>0</v>
+      </c>
+      <c r="N113" t="n">
+        <v>0</v>
+      </c>
+      <c r="O113" t="n">
+        <v>0</v>
+      </c>
+      <c r="P113" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q113" t="n">
+        <v>0</v>
+      </c>
+      <c r="R113" t="n">
+        <v>0</v>
+      </c>
+      <c r="S113" t="n">
+        <v>0</v>
+      </c>
+      <c r="T113" t="n">
+        <v>0</v>
+      </c>
+      <c r="U113" t="n">
+        <v>0</v>
+      </c>
+      <c r="V113" t="n">
+        <v>0</v>
+      </c>
+      <c r="W113" t="n">
+        <v>0</v>
+      </c>
+      <c r="X113" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y113" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA113" t="n">
+        <v>0.19497205</v>
+      </c>
+      <c r="AB113" t="n">
+        <v>0.71218324</v>
+      </c>
+      <c r="AC113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE113" t="n">
+        <v>0.09187223999999999</v>
+      </c>
+      <c r="AF113" t="n">
+        <v>0.00080586</v>
+      </c>
+      <c r="AG113" t="n">
+        <v>4.167e-05</v>
+      </c>
+      <c r="AH113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO113" t="n">
+        <v>0.00012493</v>
+      </c>
+      <c r="AP113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ113" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
           <t>F-9</t>
         </is>
       </c>
-      <c r="B113" t="n">
-        <v>0</v>
-      </c>
-      <c r="C113" t="n">
-        <v>0</v>
-      </c>
-      <c r="D113" t="n">
-        <v>0</v>
-      </c>
-      <c r="E113" t="n">
-        <v>0</v>
-      </c>
-      <c r="F113" t="n">
-        <v>0</v>
-      </c>
-      <c r="G113" t="n">
-        <v>0</v>
-      </c>
-      <c r="H113" t="n">
-        <v>0</v>
-      </c>
-      <c r="I113" t="n">
-        <v>0</v>
-      </c>
-      <c r="J113" t="n">
-        <v>0</v>
-      </c>
-      <c r="K113" t="n">
-        <v>0</v>
-      </c>
-      <c r="L113" t="n">
-        <v>0</v>
-      </c>
-      <c r="M113" t="n">
-        <v>0</v>
-      </c>
-      <c r="N113" t="n">
-        <v>0</v>
-      </c>
-      <c r="O113" t="n">
-        <v>0</v>
-      </c>
-      <c r="P113" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q113" t="n">
-        <v>0</v>
-      </c>
-      <c r="R113" t="n">
-        <v>0</v>
-      </c>
-      <c r="S113" t="n">
+      <c r="B114" t="n">
+        <v>0</v>
+      </c>
+      <c r="C114" t="n">
+        <v>0</v>
+      </c>
+      <c r="D114" t="n">
+        <v>0</v>
+      </c>
+      <c r="E114" t="n">
+        <v>0</v>
+      </c>
+      <c r="F114" t="n">
+        <v>0</v>
+      </c>
+      <c r="G114" t="n">
+        <v>0</v>
+      </c>
+      <c r="H114" t="n">
+        <v>0</v>
+      </c>
+      <c r="I114" t="n">
+        <v>0</v>
+      </c>
+      <c r="J114" t="n">
+        <v>0</v>
+      </c>
+      <c r="K114" t="n">
+        <v>0</v>
+      </c>
+      <c r="L114" t="n">
+        <v>0</v>
+      </c>
+      <c r="M114" t="n">
+        <v>0</v>
+      </c>
+      <c r="N114" t="n">
+        <v>0</v>
+      </c>
+      <c r="O114" t="n">
+        <v>0</v>
+      </c>
+      <c r="P114" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q114" t="n">
+        <v>0</v>
+      </c>
+      <c r="R114" t="n">
+        <v>0</v>
+      </c>
+      <c r="S114" t="n">
         <v>0.98648649</v>
       </c>
-      <c r="T113" t="n">
+      <c r="T114" t="n">
         <v>0.00900901</v>
       </c>
-      <c r="U113" t="n">
-        <v>0</v>
-      </c>
-      <c r="V113" t="n">
-        <v>0</v>
-      </c>
-      <c r="W113" t="n">
-        <v>0</v>
-      </c>
-      <c r="X113" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y113" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC113" t="n">
+      <c r="U114" t="n">
+        <v>0</v>
+      </c>
+      <c r="V114" t="n">
+        <v>0</v>
+      </c>
+      <c r="W114" t="n">
+        <v>0</v>
+      </c>
+      <c r="X114" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y114" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC114" t="n">
         <v>0.0045045</v>
       </c>
-      <c r="AD113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ113" t="n">
+      <c r="AD114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ114" t="n">
         <v>0</v>
       </c>
     </row>
@@ -34515,7 +34805,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>in=F-24PT, air=F-73</t>
+          <t>in=F-24PT, air=F-73T</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">

</xml_diff>